<commit_message>
Nuevo robot, finalizacion del curso basico nivel 1
</commit_message>
<xml_diff>
--- a/resources/Clase_Excel.xlsx
+++ b/resources/Clase_Excel.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\root\Downloads\Nuevo proyecto\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\root\Downloads\Nuevo proyecto\Main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F11A1B6A-2E64-43B2-8A7C-0A3952980A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6FB854D-EA0C-4944-8709-20F67955AC73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -102,14 +102,17 @@
     <t>Brasil</t>
   </si>
   <si>
-    <t>Contador</t>
+    <t>Precio</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -119,14 +122,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -159,10 +154,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -201,8 +196,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F0E051D2-F93C-4284-AD3B-911CBF92FB6F}" name="Tabla1" displayName="Tabla1" ref="A1:E30" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:E30" xr:uid="{F0E051D2-F93C-4284-AD3B-911CBF92FB6F}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F0E051D2-F93C-4284-AD3B-911CBF92FB6F}" name="Tabla1" displayName="Tabla1" ref="A1:E7" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:E7" xr:uid="{F0E051D2-F93C-4284-AD3B-911CBF92FB6F}">
     <filterColumn colId="3">
       <filters>
         <filter val="Argentina"/>
@@ -215,7 +210,7 @@
     <tableColumn id="2" xr3:uid="{A86E156F-C386-48F2-A69B-329AE06AA3B9}" name="Apellido"/>
     <tableColumn id="3" xr3:uid="{4B54360D-C891-4F93-A3E1-736BF66F78D8}" name="Direccion"/>
     <tableColumn id="4" xr3:uid="{52012AA4-2B15-4EB2-BEA2-25CFEB28E288}" name="Pais"/>
-    <tableColumn id="5" xr3:uid="{B3013459-DDBE-42EB-A0D5-94980275A91D}" name="Contador"/>
+    <tableColumn id="5" xr3:uid="{B3013459-DDBE-42EB-A0D5-94980275A91D}" name="Precio"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -518,33 +513,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" customWidth="1"/>
+    <col min="1" max="1" width="24.28515625" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" customWidth="1"/>
+    <col min="4" max="4" width="23.85546875" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -557,11 +553,11 @@
       <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E2">
-        <v>12</v>
+      <c r="E2" s="3">
+        <v>12000</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -574,11 +570,11 @@
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E3">
-        <v>15</v>
+      <c r="E3" s="3">
+        <v>15000</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -591,11 +587,11 @@
       <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E4">
-        <v>30</v>
+      <c r="E4" s="3">
+        <v>40000</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -608,11 +604,11 @@
       <c r="D5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E5">
-        <v>10</v>
+      <c r="E5" s="3">
+        <v>54000</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -625,11 +621,11 @@
       <c r="D6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E6">
-        <v>100</v>
+      <c r="E6" s="3">
+        <v>130000</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>21</v>
       </c>
@@ -642,32 +638,10 @@
       <c r="D7" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="E7" s="3">
+        <v>150000</v>
+      </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G8" s="2"/>
-    </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="17" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="18" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="19" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="20" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="21" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="22" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="23" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="24" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="25" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="26" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="27" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="28" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="29" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="30" hidden="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>